<commit_message>
Align Case 3 VAT rule with uploaded data
</commit_message>
<xml_diff>
--- a/data-mau/excel/template_invoices_mvp.xlsx
+++ b/data-mau/excel/template_invoices_mvp.xlsx
@@ -446,13 +446,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,6 +479,21 @@
           <t>total_amount</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>taxable_amount</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>vat_rate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>vat_amount</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -492,7 +510,16 @@
         <v>46037</v>
       </c>
       <c r="D2" s="3" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>1000000</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>100000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>